<commit_message>
Add newly-circulated OCTMS codes A16, A17, A18, K21 (all High risk)
Per RBI/DOR/2025-26/170 (A16-A18, KYC-related) and the Government CASA
quarterly balance-confirmation requirement (K21) — not in the original
Annexure-III set this tool was built from, confirmed via the user's live
Annexure-III sheet. Added to OCTMS_RISK in both gems.html and the Excel
calculator's risk map at High/weight 3, and bumped OCTMS_TOTAL_RISK from
302 to 314 (302 + 4x3) accordingly. Verified: gems.html via Playwright,
the workbook via a clean recalc (3,197 formulas, zero errors) and a
direct check that the denominator and new codes' ratings landed correctly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013dBYpbVDT5E5fGXRZxY5mR
</commit_message>
<xml_diff>
--- a/server/public/gems_calculator.xlsx
+++ b/server/public/gems_calculator.xlsx
@@ -52,7 +52,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="B2137" authorId="0">
+    <comment ref="B2141" authorId="0">
       <text>
         <r>
           <rPr>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="292">
   <si>
     <t xml:space="preserve">GEMS Compliance Marks Calculator</t>
   </si>
@@ -122,7 +122,7 @@
     <t xml:space="preserve">  OCRMS Risk Map   Reference table: all 67 Annexure-I parameters and their risk weights. Do not edit.</t>
   </si>
   <si>
-    <t xml:space="preserve">  OCTMS Risk Map   Reference table: all 126 Annexure-III parameters and their risk weights. Do not edit.</t>
+    <t xml:space="preserve">  OCTMS Risk Map   Reference table: all 130 Annexure-III parameters and their risk weights. Do not edit.</t>
   </si>
   <si>
     <t xml:space="preserve">NOTES</t>
@@ -509,6 +509,15 @@
     <t xml:space="preserve">A15</t>
   </si>
   <si>
+    <t xml:space="preserve">A16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A18</t>
+  </si>
+  <si>
     <t xml:space="preserve">B2</t>
   </si>
   <si>
@@ -644,6 +653,9 @@
     <t xml:space="preserve">K20</t>
   </si>
   <si>
+    <t xml:space="preserve">K21</t>
+  </si>
+  <si>
     <t xml:space="preserve">L1</t>
   </si>
   <si>
@@ -848,7 +860,7 @@
     <t xml:space="preserve">N4</t>
   </si>
   <si>
-    <t xml:space="preserve">Total risk denominator (fixed, per circular): 302</t>
+    <t xml:space="preserve">Total risk denominator (fixed, per circular): 314</t>
   </si>
   <si>
     <t xml:space="preserve">OCRMS Data — paste your WHOLE OCRMS pivot export here, starting at cell A3</t>
@@ -1775,7 +1787,7 @@
         <v>29</v>
       </c>
       <c r="B18" s="11" t="n">
-        <f aca="false">'OCTMS Data'!$B$2139</f>
+        <f aca="false">'OCTMS Data'!$B$2143</f>
         <v>1</v>
       </c>
     </row>
@@ -1784,7 +1796,7 @@
         <v>30</v>
       </c>
       <c r="B19" s="11" t="n">
-        <f aca="false">'OCTMS Data'!$B$2144</f>
+        <f aca="false">'OCTMS Data'!$B$2148</f>
         <v>1</v>
       </c>
     </row>
@@ -2798,7 +2810,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C135"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="14"/>
@@ -2991,10 +3003,10 @@
         <v>148</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C19" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3013,10 +3025,10 @@
         <v>150</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C21" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3024,10 +3036,10 @@
         <v>151</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C22" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3046,10 +3058,10 @@
         <v>153</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C24" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3068,10 +3080,10 @@
         <v>155</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C26" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3079,10 +3091,10 @@
         <v>156</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C27" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3101,10 +3113,10 @@
         <v>158</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C29" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3112,10 +3124,10 @@
         <v>159</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C30" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3145,10 +3157,10 @@
         <v>162</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C33" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3178,10 +3190,10 @@
         <v>165</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C36" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3189,10 +3201,10 @@
         <v>166</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C37" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3211,10 +3223,10 @@
         <v>168</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C39" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3222,10 +3234,10 @@
         <v>169</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C40" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3233,10 +3245,10 @@
         <v>170</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C41" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3244,10 +3256,10 @@
         <v>171</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C42" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3255,10 +3267,10 @@
         <v>172</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C43" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3266,10 +3278,10 @@
         <v>173</v>
       </c>
       <c r="B44" s="20" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C44" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3277,10 +3289,10 @@
         <v>174</v>
       </c>
       <c r="B45" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C45" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3288,10 +3300,10 @@
         <v>175</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C46" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3321,10 +3333,10 @@
         <v>178</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C49" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3332,10 +3344,10 @@
         <v>179</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C50" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3354,10 +3366,10 @@
         <v>181</v>
       </c>
       <c r="B52" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C52" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3387,10 +3399,10 @@
         <v>184</v>
       </c>
       <c r="B55" s="20" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C55" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3398,10 +3410,10 @@
         <v>185</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C56" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3409,10 +3421,10 @@
         <v>186</v>
       </c>
       <c r="B57" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C57" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3431,10 +3443,10 @@
         <v>188</v>
       </c>
       <c r="B59" s="20" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C59" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3442,10 +3454,10 @@
         <v>189</v>
       </c>
       <c r="B60" s="20" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C60" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3453,10 +3465,10 @@
         <v>190</v>
       </c>
       <c r="B61" s="20" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C61" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3464,10 +3476,10 @@
         <v>191</v>
       </c>
       <c r="B62" s="20" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C62" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3475,10 +3487,10 @@
         <v>192</v>
       </c>
       <c r="B63" s="20" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C63" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3486,10 +3498,10 @@
         <v>193</v>
       </c>
       <c r="B64" s="20" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C64" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3508,10 +3520,10 @@
         <v>195</v>
       </c>
       <c r="B66" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C66" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3541,10 +3553,10 @@
         <v>198</v>
       </c>
       <c r="B69" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C69" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3552,10 +3564,10 @@
         <v>199</v>
       </c>
       <c r="B70" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C70" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3563,10 +3575,10 @@
         <v>200</v>
       </c>
       <c r="B71" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C71" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3574,10 +3586,10 @@
         <v>201</v>
       </c>
       <c r="B72" s="20" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C72" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3618,10 +3630,10 @@
         <v>205</v>
       </c>
       <c r="B76" s="20" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C76" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3629,10 +3641,10 @@
         <v>206</v>
       </c>
       <c r="B77" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C77" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3651,10 +3663,10 @@
         <v>208</v>
       </c>
       <c r="B79" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C79" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3662,10 +3674,10 @@
         <v>209</v>
       </c>
       <c r="B80" s="20" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C80" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3673,10 +3685,10 @@
         <v>210</v>
       </c>
       <c r="B81" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C81" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3684,10 +3696,10 @@
         <v>211</v>
       </c>
       <c r="B82" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C82" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3706,10 +3718,10 @@
         <v>213</v>
       </c>
       <c r="B84" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C84" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3728,10 +3740,10 @@
         <v>215</v>
       </c>
       <c r="B86" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C86" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3739,10 +3751,10 @@
         <v>216</v>
       </c>
       <c r="B87" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C87" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3750,10 +3762,10 @@
         <v>217</v>
       </c>
       <c r="B88" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C88" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3761,10 +3773,10 @@
         <v>218</v>
       </c>
       <c r="B89" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C89" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3794,10 +3806,10 @@
         <v>221</v>
       </c>
       <c r="B92" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C92" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3805,10 +3817,10 @@
         <v>222</v>
       </c>
       <c r="B93" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C93" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3816,10 +3828,10 @@
         <v>223</v>
       </c>
       <c r="B94" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C94" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3838,10 +3850,10 @@
         <v>225</v>
       </c>
       <c r="B96" s="20" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C96" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3849,10 +3861,10 @@
         <v>226</v>
       </c>
       <c r="B97" s="20" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C97" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3860,10 +3872,10 @@
         <v>227</v>
       </c>
       <c r="B98" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C98" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3882,10 +3894,10 @@
         <v>229</v>
       </c>
       <c r="B100" s="20" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C100" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3893,10 +3905,10 @@
         <v>230</v>
       </c>
       <c r="B101" s="20" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C101" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3915,10 +3927,10 @@
         <v>232</v>
       </c>
       <c r="B103" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C103" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3926,10 +3938,10 @@
         <v>233</v>
       </c>
       <c r="B104" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C104" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3948,10 +3960,10 @@
         <v>235</v>
       </c>
       <c r="B106" s="20" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C106" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3970,10 +3982,10 @@
         <v>237</v>
       </c>
       <c r="B108" s="20" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C108" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3981,10 +3993,10 @@
         <v>238</v>
       </c>
       <c r="B109" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C109" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3992,10 +4004,10 @@
         <v>239</v>
       </c>
       <c r="B110" s="20" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C110" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4047,10 +4059,10 @@
         <v>244</v>
       </c>
       <c r="B115" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C115" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4058,10 +4070,10 @@
         <v>245</v>
       </c>
       <c r="B116" s="20" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C116" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4069,10 +4081,10 @@
         <v>246</v>
       </c>
       <c r="B117" s="20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C117" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4091,10 +4103,10 @@
         <v>248</v>
       </c>
       <c r="B119" s="20" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C119" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4102,10 +4114,10 @@
         <v>249</v>
       </c>
       <c r="B120" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C120" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4113,10 +4125,10 @@
         <v>250</v>
       </c>
       <c r="B121" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C121" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4124,10 +4136,10 @@
         <v>251</v>
       </c>
       <c r="B122" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C122" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4135,10 +4147,10 @@
         <v>252</v>
       </c>
       <c r="B123" s="20" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C123" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4146,10 +4158,10 @@
         <v>253</v>
       </c>
       <c r="B124" s="20" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C124" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4157,10 +4169,10 @@
         <v>254</v>
       </c>
       <c r="B125" s="20" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C125" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4179,10 +4191,10 @@
         <v>256</v>
       </c>
       <c r="B127" s="20" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C127" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4190,10 +4202,10 @@
         <v>257</v>
       </c>
       <c r="B128" s="20" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C128" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4201,15 +4213,59 @@
         <v>258</v>
       </c>
       <c r="B129" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="C129" s="20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="19" t="s">
+        <v>259</v>
+      </c>
+      <c r="B130" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="C129" s="20" t="n">
+      <c r="C130" s="20" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A131" s="10" t="s">
-        <v>259</v>
+      <c r="A131" s="19" t="s">
+        <v>260</v>
+      </c>
+      <c r="B131" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="C131" s="20" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="19" t="s">
+        <v>261</v>
+      </c>
+      <c r="B132" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="C132" s="20" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="19" t="s">
+        <v>262</v>
+      </c>
+      <c r="B133" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="C133" s="20" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="10" t="s">
+        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -4238,7 +4294,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="B1" s="21" t="n">
         <f aca="false">IF(B$3="",0,IFERROR(INDEX('OCRMS Risk Map'!$C:$C,MATCH(B$3,'OCRMS Risk Map'!$A:$A,0)),0))</f>
@@ -4583,7 +4639,7 @@
     </row>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="B2" s="21" t="str">
         <f aca="false">IF(B$3="","",IFERROR(INDEX('OCRMS Risk Map'!$B:$B,MATCH(B$3,'OCRMS Risk Map'!$A:$A,0)),""))</f>
@@ -4928,7 +4984,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="B3" s="23"/>
       <c r="C3" s="23"/>
@@ -5016,7 +5072,7 @@
       <c r="CG3" s="23"/>
       <c r="CH3" s="23"/>
       <c r="CJ3" s="18" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6821,7 +6877,7 @@
     </row>
     <row r="305" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A305" s="8" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B305" s="21" t="n">
         <f aca="false">IF(B1=0,0,IF(COUNTIF(B4:B303,"&gt;0")&gt;0,1,0))</f>
@@ -7166,7 +7222,7 @@
     </row>
     <row r="306" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A306" s="8" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="B306" s="21" t="n">
         <f aca="false">B305*B1</f>
@@ -7511,14 +7567,14 @@
     </row>
     <row r="309" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A309" s="6" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B309" s="7"/>
       <c r="C309" s="7"/>
     </row>
     <row r="310" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A310" s="8" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="B310" s="16" t="n">
         <f aca="false">SUM(B306:CH306)</f>
@@ -7527,7 +7583,7 @@
     </row>
     <row r="311" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A311" s="8" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="B311" s="24" t="n">
         <v>139</v>
@@ -7535,7 +7591,7 @@
     </row>
     <row r="312" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A312" s="8" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="B312" s="25" t="n">
         <f aca="false">1-(B310/B311)</f>
@@ -7544,7 +7600,7 @@
     </row>
     <row r="313" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A313" s="13" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="B313" s="14" t="n">
         <f aca="false">MIN(1,MAX(0,ROUND(B312,2)))</f>
@@ -7553,7 +7609,7 @@
     </row>
     <row r="315" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A315" s="8" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="B315" s="26" t="n">
         <f aca="false">Calculator!$B$6</f>
@@ -7562,7 +7618,7 @@
     </row>
     <row r="316" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A316" s="8" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="B316" s="16" t="n">
         <f aca="false">SUM(CJ4:CJ303)</f>
@@ -7571,7 +7627,7 @@
     </row>
     <row r="317" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A317" s="8" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="B317" s="25" t="n">
         <f aca="false">1-(B316/B315)</f>
@@ -7580,7 +7636,7 @@
     </row>
     <row r="318" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A318" s="13" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="B318" s="14" t="n">
         <f aca="false">MIN(1,MAX(0,ROUND(B317,2)))</f>
@@ -7604,7 +7660,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AL2144"/>
+  <dimension ref="A1:AL2148"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -7616,10 +7672,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="AF1" s="15" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="AG1" s="15"/>
       <c r="AH1" s="15"/>
@@ -7630,7 +7686,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="B2" s="23"/>
       <c r="C2" s="23"/>
@@ -7662,12 +7718,12 @@
       <c r="AC2" s="23"/>
       <c r="AD2" s="23"/>
       <c r="AH2" s="18" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AF3" s="8" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="AH3" s="21" t="n">
         <f aca="false">IF($AG$4=0,0,IF(INDEX($A3:$AD3,$AG$4)="",0,IF(COUNTIFS(INDEX($A$3:$AD$3,0,$AG$4),INDEX($A3:$AD3,$AG$4))=1,1,0)))</f>
@@ -7676,7 +7732,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AF4" s="10" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="AG4" s="16" t="n">
         <f aca="false">IFERROR(MATCH("BRANCH_ALPHA",$A$2:$AD$2,0),0)</f>
@@ -7689,7 +7745,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AF5" s="10" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="AG5" s="16" t="n">
         <f aca="false">IFERROR(MATCH("PARAMETER_VALUE",$A$2:$AD$2,0),0)</f>
@@ -19684,7 +19740,7 @@
     </row>
     <row r="2004" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2004" s="6" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="B2004" s="7"/>
       <c r="C2004" s="7"/>
@@ -19697,10 +19753,10 @@
         <v>60</v>
       </c>
       <c r="C2005" s="18" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="D2005" s="18" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2006" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19940,7 +19996,7 @@
     <row r="2019" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2019" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A17</f>
-        <v>B2</v>
+        <v>A16</v>
       </c>
       <c r="B2019" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C17</f>
@@ -19958,7 +20014,7 @@
     <row r="2020" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2020" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A18</f>
-        <v>B3</v>
+        <v>A17</v>
       </c>
       <c r="B2020" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C18</f>
@@ -19976,11 +20032,11 @@
     <row r="2021" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2021" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A19</f>
-        <v>B4</v>
+        <v>A18</v>
       </c>
       <c r="B2021" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C19</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2021" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2021)&gt;0,1,0))</f>
@@ -19994,7 +20050,7 @@
     <row r="2022" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2022" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A20</f>
-        <v>B5</v>
+        <v>B2</v>
       </c>
       <c r="B2022" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C20</f>
@@ -20012,11 +20068,11 @@
     <row r="2023" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2023" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A21</f>
-        <v>B6</v>
+        <v>B3</v>
       </c>
       <c r="B2023" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C21</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2023" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2023)&gt;0,1,0))</f>
@@ -20030,11 +20086,11 @@
     <row r="2024" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2024" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A22</f>
-        <v>B7</v>
+        <v>B4</v>
       </c>
       <c r="B2024" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C22</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2024" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2024)&gt;0,1,0))</f>
@@ -20048,7 +20104,7 @@
     <row r="2025" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2025" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A23</f>
-        <v>C2</v>
+        <v>B5</v>
       </c>
       <c r="B2025" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C23</f>
@@ -20066,11 +20122,11 @@
     <row r="2026" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2026" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A24</f>
-        <v>C3</v>
+        <v>B6</v>
       </c>
       <c r="B2026" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C24</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2026" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2026)&gt;0,1,0))</f>
@@ -20084,7 +20140,7 @@
     <row r="2027" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2027" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A25</f>
-        <v>C4</v>
+        <v>B7</v>
       </c>
       <c r="B2027" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C25</f>
@@ -20102,11 +20158,11 @@
     <row r="2028" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2028" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A26</f>
-        <v>C5</v>
+        <v>C2</v>
       </c>
       <c r="B2028" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C26</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2028" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2028)&gt;0,1,0))</f>
@@ -20120,11 +20176,11 @@
     <row r="2029" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2029" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A27</f>
-        <v>C6</v>
+        <v>C3</v>
       </c>
       <c r="B2029" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C27</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2029" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2029)&gt;0,1,0))</f>
@@ -20138,7 +20194,7 @@
     <row r="2030" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2030" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A28</f>
-        <v>D1</v>
+        <v>C4</v>
       </c>
       <c r="B2030" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C28</f>
@@ -20156,11 +20212,11 @@
     <row r="2031" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2031" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A29</f>
-        <v>D2</v>
+        <v>C5</v>
       </c>
       <c r="B2031" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C29</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2031" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2031)&gt;0,1,0))</f>
@@ -20174,11 +20230,11 @@
     <row r="2032" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2032" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A30</f>
-        <v>E1</v>
+        <v>C6</v>
       </c>
       <c r="B2032" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C30</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2032" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2032)&gt;0,1,0))</f>
@@ -20192,7 +20248,7 @@
     <row r="2033" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2033" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A31</f>
-        <v>E2</v>
+        <v>D1</v>
       </c>
       <c r="B2033" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C31</f>
@@ -20210,7 +20266,7 @@
     <row r="2034" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2034" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A32</f>
-        <v>F1</v>
+        <v>D2</v>
       </c>
       <c r="B2034" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C32</f>
@@ -20228,11 +20284,11 @@
     <row r="2035" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2035" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A33</f>
-        <v>F2</v>
+        <v>E1</v>
       </c>
       <c r="B2035" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C33</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2035" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2035)&gt;0,1,0))</f>
@@ -20246,7 +20302,7 @@
     <row r="2036" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2036" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A34</f>
-        <v>F3</v>
+        <v>E2</v>
       </c>
       <c r="B2036" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C34</f>
@@ -20264,7 +20320,7 @@
     <row r="2037" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2037" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A35</f>
-        <v>F4</v>
+        <v>F1</v>
       </c>
       <c r="B2037" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C35</f>
@@ -20282,11 +20338,11 @@
     <row r="2038" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2038" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A36</f>
-        <v>F5</v>
+        <v>F2</v>
       </c>
       <c r="B2038" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C36</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2038" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2038)&gt;0,1,0))</f>
@@ -20300,11 +20356,11 @@
     <row r="2039" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2039" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A37</f>
-        <v>F6</v>
+        <v>F3</v>
       </c>
       <c r="B2039" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C37</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2039" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2039)&gt;0,1,0))</f>
@@ -20318,7 +20374,7 @@
     <row r="2040" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2040" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A38</f>
-        <v>F7</v>
+        <v>F4</v>
       </c>
       <c r="B2040" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C38</f>
@@ -20336,11 +20392,11 @@
     <row r="2041" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2041" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A39</f>
-        <v>F8</v>
+        <v>F5</v>
       </c>
       <c r="B2041" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C39</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2041" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2041)&gt;0,1,0))</f>
@@ -20354,11 +20410,11 @@
     <row r="2042" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2042" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A40</f>
-        <v>F9</v>
+        <v>F6</v>
       </c>
       <c r="B2042" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C40</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2042" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2042)&gt;0,1,0))</f>
@@ -20372,11 +20428,11 @@
     <row r="2043" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2043" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A41</f>
-        <v>G1</v>
+        <v>F7</v>
       </c>
       <c r="B2043" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C41</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2043" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2043)&gt;0,1,0))</f>
@@ -20390,11 +20446,11 @@
     <row r="2044" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2044" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A42</f>
-        <v>G2</v>
+        <v>F8</v>
       </c>
       <c r="B2044" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C42</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2044" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2044)&gt;0,1,0))</f>
@@ -20408,11 +20464,11 @@
     <row r="2045" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2045" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A43</f>
-        <v>H1</v>
+        <v>F9</v>
       </c>
       <c r="B2045" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C43</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2045" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2045)&gt;0,1,0))</f>
@@ -20426,11 +20482,11 @@
     <row r="2046" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2046" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A44</f>
-        <v>I1</v>
+        <v>G1</v>
       </c>
       <c r="B2046" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C44</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C2046" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2046)&gt;0,1,0))</f>
@@ -20444,11 +20500,11 @@
     <row r="2047" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2047" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A45</f>
-        <v>I2</v>
+        <v>G2</v>
       </c>
       <c r="B2047" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C45</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2047" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2047)&gt;0,1,0))</f>
@@ -20462,11 +20518,11 @@
     <row r="2048" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2048" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A46</f>
-        <v>K1</v>
+        <v>H1</v>
       </c>
       <c r="B2048" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C46</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C2048" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2048)&gt;0,1,0))</f>
@@ -20480,7 +20536,7 @@
     <row r="2049" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2049" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A47</f>
-        <v>K2</v>
+        <v>I1</v>
       </c>
       <c r="B2049" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C47</f>
@@ -20498,7 +20554,7 @@
     <row r="2050" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2050" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A48</f>
-        <v>K3</v>
+        <v>I2</v>
       </c>
       <c r="B2050" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C48</f>
@@ -20516,11 +20572,11 @@
     <row r="2051" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2051" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A49</f>
-        <v>K4</v>
+        <v>K1</v>
       </c>
       <c r="B2051" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C49</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2051" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2051)&gt;0,1,0))</f>
@@ -20534,11 +20590,11 @@
     <row r="2052" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2052" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A50</f>
-        <v>K5</v>
+        <v>K2</v>
       </c>
       <c r="B2052" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C50</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2052" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2052)&gt;0,1,0))</f>
@@ -20552,7 +20608,7 @@
     <row r="2053" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2053" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A51</f>
-        <v>K6</v>
+        <v>K3</v>
       </c>
       <c r="B2053" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C51</f>
@@ -20570,11 +20626,11 @@
     <row r="2054" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2054" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A52</f>
-        <v>K7</v>
+        <v>K4</v>
       </c>
       <c r="B2054" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C52</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2054" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2054)&gt;0,1,0))</f>
@@ -20588,7 +20644,7 @@
     <row r="2055" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2055" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A53</f>
-        <v>K8</v>
+        <v>K5</v>
       </c>
       <c r="B2055" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C53</f>
@@ -20606,7 +20662,7 @@
     <row r="2056" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2056" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A54</f>
-        <v>K9</v>
+        <v>K6</v>
       </c>
       <c r="B2056" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C54</f>
@@ -20624,11 +20680,11 @@
     <row r="2057" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2057" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A55</f>
-        <v>K14</v>
+        <v>K7</v>
       </c>
       <c r="B2057" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C55</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2057" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2057)&gt;0,1,0))</f>
@@ -20642,11 +20698,11 @@
     <row r="2058" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2058" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A56</f>
-        <v>K15</v>
+        <v>K8</v>
       </c>
       <c r="B2058" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C56</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2058" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2058)&gt;0,1,0))</f>
@@ -20660,11 +20716,11 @@
     <row r="2059" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2059" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A57</f>
-        <v>K16</v>
+        <v>K9</v>
       </c>
       <c r="B2059" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C57</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2059" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2059)&gt;0,1,0))</f>
@@ -20678,7 +20734,7 @@
     <row r="2060" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2060" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A58</f>
-        <v>K17</v>
+        <v>K14</v>
       </c>
       <c r="B2060" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C58</f>
@@ -20696,11 +20752,11 @@
     <row r="2061" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2061" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A59</f>
-        <v>K18</v>
+        <v>K15</v>
       </c>
       <c r="B2061" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C59</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2061" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2061)&gt;0,1,0))</f>
@@ -20714,11 +20770,11 @@
     <row r="2062" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2062" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A60</f>
-        <v>K19</v>
+        <v>K16</v>
       </c>
       <c r="B2062" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C60</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2062" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2062)&gt;0,1,0))</f>
@@ -20732,11 +20788,11 @@
     <row r="2063" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2063" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A61</f>
-        <v>K20</v>
+        <v>K17</v>
       </c>
       <c r="B2063" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C61</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C2063" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2063)&gt;0,1,0))</f>
@@ -20750,11 +20806,11 @@
     <row r="2064" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2064" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A62</f>
-        <v>L1</v>
+        <v>K18</v>
       </c>
       <c r="B2064" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C62</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C2064" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2064)&gt;0,1,0))</f>
@@ -20768,11 +20824,11 @@
     <row r="2065" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2065" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A63</f>
-        <v>L2</v>
+        <v>K19</v>
       </c>
       <c r="B2065" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C63</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C2065" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2065)&gt;0,1,0))</f>
@@ -20786,11 +20842,11 @@
     <row r="2066" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2066" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A64</f>
-        <v>L3</v>
+        <v>K20</v>
       </c>
       <c r="B2066" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C64</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2066" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2066)&gt;0,1,0))</f>
@@ -20804,7 +20860,7 @@
     <row r="2067" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2067" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A65</f>
-        <v>M1</v>
+        <v>K21</v>
       </c>
       <c r="B2067" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C65</f>
@@ -20822,11 +20878,11 @@
     <row r="2068" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2068" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A66</f>
-        <v>M2</v>
+        <v>L1</v>
       </c>
       <c r="B2068" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C66</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2068" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2068)&gt;0,1,0))</f>
@@ -20840,7 +20896,7 @@
     <row r="2069" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2069" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A67</f>
-        <v>M3</v>
+        <v>L2</v>
       </c>
       <c r="B2069" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C67</f>
@@ -20858,7 +20914,7 @@
     <row r="2070" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2070" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A68</f>
-        <v>M4</v>
+        <v>L3</v>
       </c>
       <c r="B2070" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C68</f>
@@ -20876,11 +20932,11 @@
     <row r="2071" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2071" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A69</f>
-        <v>M5</v>
+        <v>M1</v>
       </c>
       <c r="B2071" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C69</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2071" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2071)&gt;0,1,0))</f>
@@ -20894,11 +20950,11 @@
     <row r="2072" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2072" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A70</f>
-        <v>M6</v>
+        <v>M2</v>
       </c>
       <c r="B2072" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C70</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2072" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2072)&gt;0,1,0))</f>
@@ -20912,11 +20968,11 @@
     <row r="2073" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2073" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A71</f>
-        <v>M7</v>
+        <v>M3</v>
       </c>
       <c r="B2073" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C71</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2073" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2073)&gt;0,1,0))</f>
@@ -20930,11 +20986,11 @@
     <row r="2074" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2074" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A72</f>
-        <v>M8</v>
+        <v>M4</v>
       </c>
       <c r="B2074" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C72</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2074" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2074)&gt;0,1,0))</f>
@@ -20948,7 +21004,7 @@
     <row r="2075" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2075" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A73</f>
-        <v>M9</v>
+        <v>M5</v>
       </c>
       <c r="B2075" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C73</f>
@@ -20966,7 +21022,7 @@
     <row r="2076" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2076" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A74</f>
-        <v>M10</v>
+        <v>M6</v>
       </c>
       <c r="B2076" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C74</f>
@@ -20984,7 +21040,7 @@
     <row r="2077" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2077" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A75</f>
-        <v>M12</v>
+        <v>M7</v>
       </c>
       <c r="B2077" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C75</f>
@@ -21002,11 +21058,11 @@
     <row r="2078" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2078" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A76</f>
-        <v>M13</v>
+        <v>M8</v>
       </c>
       <c r="B2078" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C76</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2078" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2078)&gt;0,1,0))</f>
@@ -21020,11 +21076,11 @@
     <row r="2079" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2079" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A77</f>
-        <v>M14</v>
+        <v>M9</v>
       </c>
       <c r="B2079" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C77</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2079" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2079)&gt;0,1,0))</f>
@@ -21038,7 +21094,7 @@
     <row r="2080" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2080" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A78</f>
-        <v>M15</v>
+        <v>M10</v>
       </c>
       <c r="B2080" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C78</f>
@@ -21056,11 +21112,11 @@
     <row r="2081" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2081" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A79</f>
-        <v>M17</v>
+        <v>M12</v>
       </c>
       <c r="B2081" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C79</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2081" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2081)&gt;0,1,0))</f>
@@ -21074,11 +21130,11 @@
     <row r="2082" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2082" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A80</f>
-        <v>M18</v>
+        <v>M13</v>
       </c>
       <c r="B2082" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C80</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C2082" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2082)&gt;0,1,0))</f>
@@ -21092,11 +21148,11 @@
     <row r="2083" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2083" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A81</f>
-        <v>M19</v>
+        <v>M14</v>
       </c>
       <c r="B2083" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C81</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2083" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2083)&gt;0,1,0))</f>
@@ -21110,11 +21166,11 @@
     <row r="2084" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2084" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A82</f>
-        <v>M20</v>
+        <v>M15</v>
       </c>
       <c r="B2084" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C82</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2084" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2084)&gt;0,1,0))</f>
@@ -21128,7 +21184,7 @@
     <row r="2085" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2085" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A83</f>
-        <v>M21</v>
+        <v>M17</v>
       </c>
       <c r="B2085" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C83</f>
@@ -21146,11 +21202,11 @@
     <row r="2086" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2086" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A84</f>
-        <v>M24</v>
+        <v>M18</v>
       </c>
       <c r="B2086" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C84</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2086" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2086)&gt;0,1,0))</f>
@@ -21164,7 +21220,7 @@
     <row r="2087" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2087" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A85</f>
-        <v>M25</v>
+        <v>M19</v>
       </c>
       <c r="B2087" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C85</f>
@@ -21182,11 +21238,11 @@
     <row r="2088" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2088" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A86</f>
-        <v>M26</v>
+        <v>M20</v>
       </c>
       <c r="B2088" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C86</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2088" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2088)&gt;0,1,0))</f>
@@ -21200,11 +21256,11 @@
     <row r="2089" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2089" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A87</f>
-        <v>M27</v>
+        <v>M21</v>
       </c>
       <c r="B2089" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C87</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2089" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2089)&gt;0,1,0))</f>
@@ -21218,11 +21274,11 @@
     <row r="2090" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2090" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A88</f>
-        <v>M28</v>
+        <v>M24</v>
       </c>
       <c r="B2090" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C88</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2090" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2090)&gt;0,1,0))</f>
@@ -21236,11 +21292,11 @@
     <row r="2091" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2091" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A89</f>
-        <v>M29</v>
+        <v>M25</v>
       </c>
       <c r="B2091" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C89</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2091" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2091)&gt;0,1,0))</f>
@@ -21254,7 +21310,7 @@
     <row r="2092" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2092" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A90</f>
-        <v>M30</v>
+        <v>M26</v>
       </c>
       <c r="B2092" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C90</f>
@@ -21272,7 +21328,7 @@
     <row r="2093" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2093" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A91</f>
-        <v>M31</v>
+        <v>M27</v>
       </c>
       <c r="B2093" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C91</f>
@@ -21290,11 +21346,11 @@
     <row r="2094" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2094" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A92</f>
-        <v>M32</v>
+        <v>M28</v>
       </c>
       <c r="B2094" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C92</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2094" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2094)&gt;0,1,0))</f>
@@ -21308,11 +21364,11 @@
     <row r="2095" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2095" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A93</f>
-        <v>M33</v>
+        <v>M29</v>
       </c>
       <c r="B2095" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C93</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2095" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2095)&gt;0,1,0))</f>
@@ -21326,11 +21382,11 @@
     <row r="2096" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2096" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A94</f>
-        <v>M34</v>
+        <v>M30</v>
       </c>
       <c r="B2096" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C94</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2096" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2096)&gt;0,1,0))</f>
@@ -21344,7 +21400,7 @@
     <row r="2097" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2097" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A95</f>
-        <v>M35</v>
+        <v>M31</v>
       </c>
       <c r="B2097" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C95</f>
@@ -21362,11 +21418,11 @@
     <row r="2098" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2098" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A96</f>
-        <v>M36</v>
+        <v>M32</v>
       </c>
       <c r="B2098" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C96</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2098" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2098)&gt;0,1,0))</f>
@@ -21380,11 +21436,11 @@
     <row r="2099" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2099" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A97</f>
-        <v>M37</v>
+        <v>M33</v>
       </c>
       <c r="B2099" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C97</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2099" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2099)&gt;0,1,0))</f>
@@ -21398,11 +21454,11 @@
     <row r="2100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2100" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A98</f>
-        <v>M38</v>
+        <v>M34</v>
       </c>
       <c r="B2100" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C98</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2100" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2100)&gt;0,1,0))</f>
@@ -21416,7 +21472,7 @@
     <row r="2101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2101" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A99</f>
-        <v>M39</v>
+        <v>M35</v>
       </c>
       <c r="B2101" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C99</f>
@@ -21434,11 +21490,11 @@
     <row r="2102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2102" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A100</f>
-        <v>M40</v>
+        <v>M36</v>
       </c>
       <c r="B2102" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C100</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C2102" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2102)&gt;0,1,0))</f>
@@ -21452,11 +21508,11 @@
     <row r="2103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2103" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A101</f>
-        <v>M41</v>
+        <v>M37</v>
       </c>
       <c r="B2103" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C101</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2103" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2103)&gt;0,1,0))</f>
@@ -21470,7 +21526,7 @@
     <row r="2104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2104" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A102</f>
-        <v>M42</v>
+        <v>M38</v>
       </c>
       <c r="B2104" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C102</f>
@@ -21488,11 +21544,11 @@
     <row r="2105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2105" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A103</f>
-        <v>M43</v>
+        <v>M39</v>
       </c>
       <c r="B2105" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C103</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2105" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2105)&gt;0,1,0))</f>
@@ -21506,11 +21562,11 @@
     <row r="2106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2106" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A104</f>
-        <v>M44</v>
+        <v>M40</v>
       </c>
       <c r="B2106" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C104</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2106" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2106)&gt;0,1,0))</f>
@@ -21524,7 +21580,7 @@
     <row r="2107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2107" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A105</f>
-        <v>M45</v>
+        <v>M41</v>
       </c>
       <c r="B2107" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C105</f>
@@ -21542,11 +21598,11 @@
     <row r="2108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2108" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A106</f>
-        <v>M46</v>
+        <v>M42</v>
       </c>
       <c r="B2108" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C106</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2108" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2108)&gt;0,1,0))</f>
@@ -21560,7 +21616,7 @@
     <row r="2109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2109" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A107</f>
-        <v>M47</v>
+        <v>M43</v>
       </c>
       <c r="B2109" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C107</f>
@@ -21578,11 +21634,11 @@
     <row r="2110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2110" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A108</f>
-        <v>M48</v>
+        <v>M44</v>
       </c>
       <c r="B2110" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C108</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2110" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2110)&gt;0,1,0))</f>
@@ -21596,11 +21652,11 @@
     <row r="2111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2111" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A109</f>
-        <v>M49</v>
+        <v>M45</v>
       </c>
       <c r="B2111" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C109</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2111" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2111)&gt;0,1,0))</f>
@@ -21614,11 +21670,11 @@
     <row r="2112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2112" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A110</f>
-        <v>M50</v>
+        <v>M46</v>
       </c>
       <c r="B2112" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C110</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2112" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2112)&gt;0,1,0))</f>
@@ -21632,7 +21688,7 @@
     <row r="2113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2113" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A111</f>
-        <v>M51</v>
+        <v>M47</v>
       </c>
       <c r="B2113" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C111</f>
@@ -21650,7 +21706,7 @@
     <row r="2114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2114" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A112</f>
-        <v>M52</v>
+        <v>M48</v>
       </c>
       <c r="B2114" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C112</f>
@@ -21668,7 +21724,7 @@
     <row r="2115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2115" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A113</f>
-        <v>M53</v>
+        <v>M49</v>
       </c>
       <c r="B2115" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C113</f>
@@ -21686,7 +21742,7 @@
     <row r="2116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2116" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A114</f>
-        <v>M54</v>
+        <v>M50</v>
       </c>
       <c r="B2116" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C114</f>
@@ -21704,11 +21760,11 @@
     <row r="2117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2117" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A115</f>
-        <v>M55</v>
+        <v>M51</v>
       </c>
       <c r="B2117" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C115</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2117" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2117)&gt;0,1,0))</f>
@@ -21722,11 +21778,11 @@
     <row r="2118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2118" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A116</f>
-        <v>M56</v>
+        <v>M52</v>
       </c>
       <c r="B2118" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C116</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2118" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2118)&gt;0,1,0))</f>
@@ -21740,11 +21796,11 @@
     <row r="2119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2119" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A117</f>
-        <v>M57</v>
+        <v>M53</v>
       </c>
       <c r="B2119" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C117</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2119" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2119)&gt;0,1,0))</f>
@@ -21758,7 +21814,7 @@
     <row r="2120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2120" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A118</f>
-        <v>M58</v>
+        <v>M54</v>
       </c>
       <c r="B2120" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C118</f>
@@ -21776,11 +21832,11 @@
     <row r="2121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2121" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A119</f>
-        <v>M59</v>
+        <v>M55</v>
       </c>
       <c r="B2121" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C119</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2121" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2121)&gt;0,1,0))</f>
@@ -21794,11 +21850,11 @@
     <row r="2122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2122" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A120</f>
-        <v>M60</v>
+        <v>M56</v>
       </c>
       <c r="B2122" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C120</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2122" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2122)&gt;0,1,0))</f>
@@ -21812,11 +21868,11 @@
     <row r="2123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2123" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A121</f>
-        <v>M61</v>
+        <v>M57</v>
       </c>
       <c r="B2123" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C121</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2123" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2123)&gt;0,1,0))</f>
@@ -21830,11 +21886,11 @@
     <row r="2124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2124" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A122</f>
-        <v>M62</v>
+        <v>M58</v>
       </c>
       <c r="B2124" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C122</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2124" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2124)&gt;0,1,0))</f>
@@ -21848,11 +21904,11 @@
     <row r="2125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2125" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A123</f>
-        <v>M63</v>
+        <v>M59</v>
       </c>
       <c r="B2125" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C123</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2125" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2125)&gt;0,1,0))</f>
@@ -21866,11 +21922,11 @@
     <row r="2126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2126" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A124</f>
-        <v>M64</v>
+        <v>M60</v>
       </c>
       <c r="B2126" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C124</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2126" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2126)&gt;0,1,0))</f>
@@ -21884,11 +21940,11 @@
     <row r="2127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2127" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A125</f>
-        <v>M65</v>
+        <v>M61</v>
       </c>
       <c r="B2127" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C125</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2127" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2127)&gt;0,1,0))</f>
@@ -21902,7 +21958,7 @@
     <row r="2128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2128" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A126</f>
-        <v>N1</v>
+        <v>M62</v>
       </c>
       <c r="B2128" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C126</f>
@@ -21920,11 +21976,11 @@
     <row r="2129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2129" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A127</f>
-        <v>N2</v>
+        <v>M63</v>
       </c>
       <c r="B2129" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C127</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2129" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2129)&gt;0,1,0))</f>
@@ -21938,11 +21994,11 @@
     <row r="2130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2130" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A128</f>
-        <v>N3</v>
+        <v>M64</v>
       </c>
       <c r="B2130" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C128</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C2130" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2130)&gt;0,1,0))</f>
@@ -21956,11 +22012,11 @@
     <row r="2131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2131" s="26" t="str">
         <f aca="false">'OCTMS Risk Map'!A129</f>
-        <v>N4</v>
+        <v>M65</v>
       </c>
       <c r="B2131" s="28" t="n">
         <f aca="false">'OCTMS Risk Map'!C129</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C2131" s="21" t="n">
         <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2131)&gt;0,1,0))</f>
@@ -21971,90 +22027,162 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2133" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2133" s="5" t="s">
-        <v>285</v>
+    <row r="2132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2132" s="26" t="str">
+        <f aca="false">'OCTMS Risk Map'!A130</f>
+        <v>N1</v>
+      </c>
+      <c r="B2132" s="28" t="n">
+        <f aca="false">'OCTMS Risk Map'!C130</f>
+        <v>3</v>
+      </c>
+      <c r="C2132" s="21" t="n">
+        <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2132)&gt;0,1,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D2132" s="21" t="n">
+        <f aca="false">C2132*B2132</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2133" s="26" t="str">
+        <f aca="false">'OCTMS Risk Map'!A131</f>
+        <v>N2</v>
+      </c>
+      <c r="B2133" s="28" t="n">
+        <f aca="false">'OCTMS Risk Map'!C131</f>
+        <v>3</v>
+      </c>
+      <c r="C2133" s="21" t="n">
+        <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2133)&gt;0,1,0))</f>
+        <v>0</v>
       </c>
       <c r="D2133" s="21" t="n">
-        <f aca="false">IF($AG$5=0,0,SUMPRODUCT((INDEX($A$3:$AD$2002,0,$AG$5)&lt;&gt;"")*ISNA(MATCH(INDEX($A$3:$AD$2002,0,$AG$5),$A$2006:$A$2131,0))))</f>
+        <f aca="false">C2133*B2133</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2134" s="26" t="str">
+        <f aca="false">'OCTMS Risk Map'!A132</f>
+        <v>N3</v>
+      </c>
+      <c r="B2134" s="28" t="n">
+        <f aca="false">'OCTMS Risk Map'!C132</f>
+        <v>3</v>
+      </c>
+      <c r="C2134" s="21" t="n">
+        <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2134)&gt;0,1,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D2134" s="21" t="n">
+        <f aca="false">C2134*B2134</f>
         <v>0</v>
       </c>
     </row>
     <row r="2135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2135" s="6" t="s">
-        <v>286</v>
-      </c>
-      <c r="B2135" s="7"/>
-      <c r="C2135" s="7"/>
-    </row>
-    <row r="2136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2136" s="8" t="s">
-        <v>267</v>
-      </c>
-      <c r="B2136" s="16" t="n">
-        <f aca="false">SUM(D2006:D2131)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2137" s="8" t="s">
-        <v>268</v>
-      </c>
-      <c r="B2137" s="24" t="n">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="2138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2138" s="8" t="s">
-        <v>269</v>
-      </c>
-      <c r="B2138" s="25" t="n">
-        <f aca="false">1-(B2136/B2137)</f>
-        <v>1</v>
+      <c r="A2135" s="26" t="str">
+        <f aca="false">'OCTMS Risk Map'!A133</f>
+        <v>N4</v>
+      </c>
+      <c r="B2135" s="28" t="n">
+        <f aca="false">'OCTMS Risk Map'!C133</f>
+        <v>3</v>
+      </c>
+      <c r="C2135" s="21" t="n">
+        <f aca="false">IF($AG$5=0,0,IF(COUNTIF(INDEX($A$3:$AD$2002,0,$AG$5),A2135)&gt;0,1,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D2135" s="21" t="n">
+        <f aca="false">C2135*B2135</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2137" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2137" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D2137" s="21" t="n">
+        <f aca="false">IF($AG$5=0,0,SUMPRODUCT((INDEX($A$3:$AD$2002,0,$AG$5)&lt;&gt;"")*ISNA(MATCH(INDEX($A$3:$AD$2002,0,$AG$5),$A$2006:$A$2135,0))))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="2139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2139" s="13" t="s">
-        <v>270</v>
-      </c>
-      <c r="B2139" s="14" t="n">
-        <f aca="false">MIN(1,MAX(0,ROUND(B2138,2)))</f>
-        <v>1</v>
+      <c r="A2139" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="B2139" s="7"/>
+      <c r="C2139" s="7"/>
+    </row>
+    <row r="2140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2140" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="B2140" s="16" t="n">
+        <f aca="false">SUM(D2006:D2135)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="2141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2141" s="8" t="s">
-        <v>271</v>
-      </c>
-      <c r="B2141" s="26" t="n">
+        <v>272</v>
+      </c>
+      <c r="B2141" s="24" t="n">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="2142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2142" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B2142" s="25" t="n">
+        <f aca="false">1-(B2140/B2141)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2143" s="13" t="s">
+        <v>274</v>
+      </c>
+      <c r="B2143" s="14" t="n">
+        <f aca="false">MIN(1,MAX(0,ROUND(B2142,2)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2145" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="B2145" s="26" t="n">
         <f aca="false">Calculator!$B$6</f>
         <v>55</v>
       </c>
     </row>
-    <row r="2142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2142" s="8" t="s">
-        <v>287</v>
-      </c>
-      <c r="B2142" s="16" t="n">
+    <row r="2146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2146" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="B2146" s="16" t="n">
         <f aca="false">SUM(AH3:AH2002)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="2143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2143" s="8" t="s">
-        <v>273</v>
-      </c>
-      <c r="B2143" s="25" t="n">
-        <f aca="false">1-(B2142/B2141)</f>
+    <row r="2147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2147" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="B2147" s="25" t="n">
+        <f aca="false">1-(B2146/B2145)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="2144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2144" s="13" t="s">
-        <v>274</v>
-      </c>
-      <c r="B2144" s="14" t="n">
-        <f aca="false">MIN(1,MAX(0,ROUND(B2143,2)))</f>
+    <row r="2148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2148" s="13" t="s">
+        <v>278</v>
+      </c>
+      <c r="B2148" s="14" t="n">
+        <f aca="false">MIN(1,MAX(0,ROUND(B2147,2)))</f>
         <v>1</v>
       </c>
     </row>

</xml_diff>